<commit_message>
Refactor human agent data structure and enhance schema documentation
- Updated `human_agents.json` to replace `count_of_rles` with `count_of_roles`, improving clarity in role tracking.
- Enhanced the `substrate-report.html` and `test-results.md` to reflect the updated metrics and results, ensuring accurate reporting of human agent roles.
- Revised `english-specification.md` to include detailed descriptions of input fields and calculated fields for workflows, workflow steps, and roles, improving usability and understanding of the schema.
- Adjusted HTML reports to align with the new structure, enhancing overall readability and user experience.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -145,6 +145,191 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Human-readable name for the workflow. Maps to dct:title per Dublin Core.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Detailed description of the workflow purpose and scope. Maps to dct:description per Dublin Core.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Date the workflow was created. Maps to dct:created per Dublin Core.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Date the workflow was last modified. Maps to dct:modified. Used to identify stale workflows per NTWF CQ5.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>External reference identifier (e.g., ticket number). Maps to dct:identifier. Join key to operational systems.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Steps contained in this workflow. Inverse of IsStepOf. Maps to ntwf:hasStep.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Count of steps in this workflow. Aggregation over IsStepOf relationship.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Human-readable name for the step. Maps to rdfs:label.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Ordinal position in workflow sequence. Maps to ntwf:sequencePosition (functional). Supports positional ordering queries.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Whether this step requires a human agent. Maps to ntwf:requiresHumanApproval. Answers NTWF CQ3.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Parent workflow containing this step. Inverse of WorkflowSteps. Maps to ntwf:isStepOf.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Role responsible for this step. Maps to ntwf:assignedRole (functional). Implements role-agent separation.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of parent workflow title.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of parent workflow description.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of parent workflow external identifier.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of assigned role label.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of assigned role comment/description.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of agent currently filling the assigned role.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Human-readable name for the role. Maps to rdfs:label.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Description of the role's responsibilities. Maps to rdfs:comment.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Agent currently filling this role. Maps to ntwf:filledBy. The change-management triple - update this when personnel change.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Steps assigned to this role. Inverse of AssignedRole.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Count of workflow steps assigned to this role.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of agent name (foaf:name) filling this role.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Denormalized lookup of agent email (foaf:mbox) filling this role.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Full name of the person. Maps to foaf:name per FOAF ontology.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Email address of the person. Maps to foaf:mbox per FOAF ontology. Used for contact and identity resolution.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Roles filled by this agent. Inverse of FilledBy.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Count of roles currently filled by this agent.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -533,6 +718,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -789,6 +975,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -951,6 +1138,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -960,14 +1148,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -993,7 +1181,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CountOfRles</t>
+          <t>CountOfRoles</t>
         </is>
       </c>
     </row>
@@ -1025,17 +1213,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>james-okafor</t>
+          <t>maria-gonzalez</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>James Okafor</t>
+          <t>Maria Gonzalez</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>james.okafor@specialsolutions.example</t>
+          <t>maria.gonzalez@specialsolutions.example</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -1043,7 +1231,155 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>james-okafor</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>James Okafor</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>james.okafor@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>maria-gonzalez</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Maria Gonzalez</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>maria.gonzalez@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>james-okafor</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>James Okafor</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>james.okafor@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>maria-gonzalez</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Maria Gonzalez</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>maria.gonzalez@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>james-okafor</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>James Okafor</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>james.okafor@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>maria-gonzalez</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Maria Gonzalez</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>maria.gonzalez@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>james-okafor</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>James Okafor</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>james.okafor@specialsolutions.example</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance JTO v3 Rulebook Specification and Update Schema Documentation
- Revised `english-specification.md` to improve clarity and detail for workflows, workflow steps, roles, and human agents, including updated descriptions for input and calculated fields.
- Added a new `DelegatesTo` field in `effortless-rulebook.json` to support escalation processes for roles, enhancing the schema's functionality.
- Updated HTML reports and test results to reflect changes in the schema, ensuring accurate representation of metrics and improved readability.
- Cleaned up redundant entries in JSON test answer files for human agents and roles, streamlining data integrity and validation processes.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -296,6 +296,11 @@
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Denormalized lookup of agent email (foaf:mbox) filling this role.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Role to escalate to when this role's agent is unavailable. Maps to ntwf:delegatesTo. Enables delegation chain queries.</t>
       </text>
     </comment>
   </commentList>
@@ -985,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -996,6 +1001,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1039,6 +1045,11 @@
           <t>FilledByMBox</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>DelegatesTo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1079,6 +1090,7 @@
           <t>maria.gonzalez@specialsolutions.example</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1107,6 +1119,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1135,6 +1148,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1148,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1213,168 +1227,21 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>maria-gonzalez</t>
+          <t>james-okafor</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Maria Gonzalez</t>
+          <t>James Okafor</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>maria.gonzalez@specialsolutions.example</t>
+          <t>james.okafor@specialsolutions.example</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>james-okafor</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>James Okafor</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>james.okafor@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>maria-gonzalez</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Maria Gonzalez</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>maria.gonzalez@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>james-okafor</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>James Okafor</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>james.okafor@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>maria-gonzalez</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Maria Gonzalez</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>maria.gonzalez@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>james-okafor</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>James Okafor</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>james.okafor@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>maria-gonzalez</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Maria Gonzalez</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>maria.gonzalez@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>james-okafor</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>James Okafor</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>james.okafor@specialsolutions.example</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Jessica's Ontology Series-v3 Rulebook and Enhance Role Delegation Features
- Revised `english-specification.md` to clarify the structure and calculations for workflows, workflow steps, roles, and human agents, improving overall documentation.
- Added new fields `DelegatesTo` and `DelegatedToBy` in `effortless-rulebook.json` to support role escalation and delegation processes, enhancing schema functionality.
- Updated HTML reports and test results to reflect the new schema changes, ensuring accurate representation of metrics and improved readability.
- Cleaned up JSON test answer files for roles, streamlining data integrity and validation processes.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -290,17 +290,17 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
+        <t>Role to escalate to when this role's agent is unavailable. Maps to ntwf:delegatesTo. Enables delegation chain queries.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
         <t>Denormalized lookup of agent name (foaf:name) filling this role.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Denormalized lookup of agent email (foaf:mbox) filling this role.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Role to escalate to when this role's agent is unavailable. Maps to ntwf:delegatesTo. Enables delegation chain queries.</t>
       </text>
     </comment>
   </commentList>
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -999,9 +999,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1037,17 +1039,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>DelegatesTo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Label_from_DelegatesTo</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>FilledByName</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>FilledByMBox</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>DelegatesTo</t>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DelegatedToBy</t>
         </is>
       </c>
     </row>
@@ -1082,15 +1094,25 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>vp-engineering</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>VP Engineering</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Maria Gonzalez</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>maria.gonzalez@specialsolutions.example</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1120,6 +1142,8 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1149,6 +1173,78 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>vp-engineering</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>VP Engineering</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Secondary role in delegation chain. Escalation from Release Manager when primary agent unavailable. Article CQ6.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>cto</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>release-manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>cto</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Final role in delegation chain. Ultimate authority for release decisions. Article CQ6.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>vp-engineering</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update rulebook paths and enhance error handling in orchestration scripts
- Updated references in `active-domain.txt` to switch the active domain to "customer-fullname."
- Refactored `orchestrate.sh` to improve error handling for missing or incorrect rulebook paths, ensuring clearer error messages.
- Adjusted `substrate-report.html` to reflect updated test results and rulebook statistics.
- Modified various JSON and SQL files to align with the new project structure and naming conventions, including updates to the rulebook and generated files.
- Enhanced documentation for better clarity and maintainability across the project.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +494,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -523,12 +521,13 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>jane-smith-email-com</t>
-        </is>
-      </c>
-      <c r="B2" s="3">
-        <f>SUBSTITUTE($C2, "@", "-")</f>
-        <v/>
+          <t>cust0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CUST0001</t>
+        </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -537,7 +536,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Bobby</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -553,12 +552,13 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>john-doe-email-com</t>
-        </is>
-      </c>
-      <c r="B3" s="3">
-        <f>SUBSTITUTE($C3, "@", "-")</f>
-        <v/>
+          <t>cust0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CUST0002</t>
+        </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Jimmy</t>
+          <t>John</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -583,12 +583,13 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>emily-jones-email-com</t>
-        </is>
-      </c>
-      <c r="B4" s="3">
-        <f>SUBSTITUTE($C4, "@", "-")</f>
-        <v/>
+          <t>cust0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CUST0003</t>
+        </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -597,7 +598,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Emily</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -614,349 +615,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBVersionId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>BaseId</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CommitDate</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IsPublished</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBCustomizationId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>SQLCode</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SQLTarget</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CustomizationType</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema-sql</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema.sql</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Customize Schema</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE SCHEMA - User-defined tables and schema modifications
--- ============================================================================
--- This file is for YOUR custom schema changes that should persist across
--- regeneration of the base ERB files.
---
--- USE THIS FILE FOR:
---   - Additional tables not defined in the rulebook
---   - Extra columns on existing tables (ALTER TABLE)
---   - Custom indexes for performance tuning
---   - Custom constraints or triggers
---
--- IMPORTANT:
---   - This file runs AFTER 01-drop-and-create-tables.sql
---   - The base tables already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom schema changes go here:
-</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions-sql</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions.sql</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Customize Functions</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE FUNCTIONS - User-defined calculation functions
--- ============================================================================
--- This file is for YOUR custom PostgreSQL functions that should persist
--- across regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 02-create-functions.sql
---   - Base ERB calc functions already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom functions go here:
-</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Functions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views-sql</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views.sql</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Customize Views</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE VIEWS - User-defined views and view extensions
--- ============================================================================
--- This file is for YOUR custom views that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 03-create-views.sql
---   - All base vw_* views already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom views go here:
-</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Views</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls-sql</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls.sql</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Customize Policies (RLS)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE POLICIES - User-defined Row Level Security policies
--- ============================================================================
--- This file is for YOUR custom RLS policies that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 04-create-policies.sql
---   - Base RLS policies already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom policies go here:
-</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data-sql</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data.sql</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Customize Data (Seeds / Migrations)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE DATA - User-defined seed data and data migrations
--- ============================================================================
--- This file is for YOUR custom seed data that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 05-insert-data.sql
---   - Base seed data already exists when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom data inserts go here:
-</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update PostgreSQL substrate reports and enhance orchestration scripts
- Modified `substrate-report.html` for the effortless-postgres substrate to reflect updated test results, showing a score of 0.0% with 0/6 tests passed.
- Adjusted `all-tests-results.md` to summarize the new test outcomes, indicating a total of 2 substrates tested with an overall score of 50.0%.
- Updated orchestration scripts to improve error handling and ensure accurate reporting of test results.
- Added new PostgreSQL scripts for schema creation and data insertion, supporting the updated project structure for the customer-fullname example.
- Enhanced documentation for better clarity and maintainability across the project.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -521,13 +521,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>cust0001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CUST0001</t>
-        </is>
+          <t>jane-smith-email-com</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>SUBSTITUTE($C2, "@", "-")</f>
+        <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -536,7 +535,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>Bobby</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -552,13 +551,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>cust0002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>CUST0002</t>
-        </is>
+          <t>john-doe-email-com</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>SUBSTITUTE($C3, "@", "-")</f>
+        <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -567,7 +565,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -583,13 +581,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>cust0003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>CUST0003</t>
-        </is>
+          <t>emily-jones-email-com</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>SUBSTITUTE($C4, "@", "-")</f>
+        <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -598,7 +595,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Emily</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add Domain Switcher Component and Update UI
- Introduced a new DomainSwitcher component for improved domain selection in the admin portal.
- Updated RoleTopBar to utilize the DomainSwitcher, enhancing user experience by replacing the previous dropdown.
- Enhanced CSS styles for the domain switcher and related UI elements for better visual consistency.
- Adjusted Developer and Viewer screens to incorporate domain card designs, displaying logos and descriptions for better clarity.
- Added a scheduled tasks lock file to manage session states.

This commit aims to streamline domain management and improve the overall user interface in the admin portal.
</commit_message>
<xml_diff>
--- a/execution-substrates/xlsx/rulebook.xlsx
+++ b/execution-substrates/xlsx/rulebook.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Bobby</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="F2" s="3">
-        <f>$E2 &amp; ", " &amp; $D2</f>
+        <f>$D2 &amp; " " &amp; $E2</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="F3" s="3">
-        <f>$E3 &amp; ", " &amp; $D3</f>
+        <f>$D3 &amp; " " &amp; $E3</f>
         <v/>
       </c>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="F4" s="3">
-        <f>$E4 &amp; ", " &amp; $D4</f>
+        <f>$D4 &amp; " " &amp; $E4</f>
         <v/>
       </c>
     </row>

</xml_diff>